<commit_message>
ANTES DE VARIABLE ANCLA
</commit_message>
<xml_diff>
--- a/Indc WDI_V6.xlsx
+++ b/Indc WDI_V6.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\messi\OneDrive\Escritorio\escuela\Servicio Social\Python\PCA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00E8B7BE-D6EA-43EF-84A3-146F51BB8073}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{787244A7-7F0A-470F-B5E5-D551E4F2C9B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="3" activeTab="4" xr2:uid="{D86699F4-EEE8-4FD6-B0D7-CE6A5D28E5C9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D86699F4-EEE8-4FD6-B0D7-CE6A5D28E5C9}"/>
   </bookViews>
   <sheets>
     <sheet name="GDP growth (annual %)" sheetId="25" r:id="rId1"/>
@@ -3288,6 +3288,14 @@
         <f>L2</f>
         <v>4568.56640625</v>
       </c>
+      <c r="V2" s="5">
+        <f>L2</f>
+        <v>4568.56640625</v>
+      </c>
+      <c r="W2" s="5">
+        <f>L2</f>
+        <v>4568.56640625</v>
+      </c>
       <c r="X2" s="5">
         <f>L2</f>
         <v>4568.56640625</v>
@@ -3474,6 +3482,10 @@
       <c r="U5">
         <v>5561.72998046875</v>
       </c>
+      <c r="V5" s="5">
+        <f>U5</f>
+        <v>5561.72998046875</v>
+      </c>
       <c r="W5">
         <v>6021.3984375</v>
       </c>
@@ -4235,6 +4247,10 @@
       <c r="V16">
         <v>259.26324462890602</v>
       </c>
+      <c r="W16" s="5">
+        <f>V16</f>
+        <v>259.26324462890602</v>
+      </c>
       <c r="X16" s="5">
         <f>V16</f>
         <v>259.26324462890602</v>
@@ -4274,6 +4290,10 @@
         <v>387.17062377929699</v>
       </c>
       <c r="V17">
+        <v>395.34167480468801</v>
+      </c>
+      <c r="W17" s="5">
+        <f>V17</f>
         <v>395.34167480468801</v>
       </c>
       <c r="X17" s="5">
@@ -5658,6 +5678,10 @@
       <c r="U2">
         <v>1.82570004463196</v>
       </c>
+      <c r="V2" s="5">
+        <f>W2</f>
+        <v>1.8550900220871001</v>
+      </c>
       <c r="W2">
         <v>1.8550900220871001</v>
       </c>
@@ -5847,6 +5871,10 @@
       <c r="U5">
         <v>3.1967999935150102</v>
       </c>
+      <c r="V5" s="5">
+        <f>W5</f>
+        <v>3.3064498901367201</v>
+      </c>
       <c r="W5">
         <v>3.3064498901367201</v>
       </c>
@@ -6658,6 +6686,10 @@
       <c r="V16">
         <v>0.645579993724823</v>
       </c>
+      <c r="W16" s="5">
+        <f>V16</f>
+        <v>0.645579993724823</v>
+      </c>
       <c r="X16" s="5">
         <v>0.63812401294708199</v>
       </c>
@@ -6697,6 +6729,10 @@
         <v>0.27129000425338701</v>
       </c>
       <c r="V17">
+        <v>0.28068000078201299</v>
+      </c>
+      <c r="W17" s="5">
+        <f>V17</f>
         <v>0.28068000078201299</v>
       </c>
       <c r="X17" s="5">
@@ -18494,6 +18530,14 @@
       <c r="U2" s="5">
         <v>12.7</v>
       </c>
+      <c r="V2" s="5">
+        <f>U2</f>
+        <v>12.7</v>
+      </c>
+      <c r="W2" s="5">
+        <f>T2</f>
+        <v>12.7</v>
+      </c>
       <c r="X2" s="5">
         <f>T2</f>
         <v>12.7</v>
@@ -18632,6 +18676,14 @@
       <c r="U4">
         <v>12.5</v>
       </c>
+      <c r="V4" s="5">
+        <f>U4</f>
+        <v>12.5</v>
+      </c>
+      <c r="W4" s="5">
+        <f>U4</f>
+        <v>12.5</v>
+      </c>
       <c r="X4" s="5">
         <f>U4</f>
         <v>12.5</v>
@@ -18695,6 +18747,10 @@
       <c r="V5">
         <v>11.7</v>
       </c>
+      <c r="W5" s="5">
+        <f>V5</f>
+        <v>11.7</v>
+      </c>
       <c r="X5" s="5">
         <f>V5</f>
         <v>11.7</v>
@@ -18898,6 +18954,10 @@
       <c r="V8">
         <v>12</v>
       </c>
+      <c r="W8" s="5">
+        <f>V8</f>
+        <v>12</v>
+      </c>
       <c r="X8" s="5">
         <f>V8</f>
         <v>12</v>
@@ -19687,6 +19747,14 @@
         <f>O20</f>
         <v>11</v>
       </c>
+      <c r="V20" s="5">
+        <f>U20</f>
+        <v>11</v>
+      </c>
+      <c r="W20" s="5">
+        <f>V20</f>
+        <v>11</v>
+      </c>
       <c r="X20" s="5">
         <f>O20</f>
         <v>11</v>
@@ -19997,6 +20065,10 @@
       <c r="V25">
         <v>24.7</v>
       </c>
+      <c r="W25" s="5">
+        <f>V25</f>
+        <v>24.7</v>
+      </c>
       <c r="X25">
         <v>22.5</v>
       </c>
@@ -20124,6 +20196,14 @@
         <v>9</v>
       </c>
       <c r="U27">
+        <v>9.4</v>
+      </c>
+      <c r="V27" s="5">
+        <f>U27</f>
+        <v>9.4</v>
+      </c>
+      <c r="W27" s="5">
+        <f>V27</f>
         <v>9.4</v>
       </c>
       <c r="X27" s="5">
@@ -20807,6 +20887,14 @@
         <f>T2</f>
         <v>1</v>
       </c>
+      <c r="V2" s="5">
+        <f>U2</f>
+        <v>1</v>
+      </c>
+      <c r="W2" s="5">
+        <f>T2</f>
+        <v>1</v>
+      </c>
       <c r="X2" s="5">
         <f>T2</f>
         <v>1</v>
@@ -20945,6 +21033,14 @@
       <c r="U4">
         <v>0.7</v>
       </c>
+      <c r="V4" s="5">
+        <f>U4</f>
+        <v>0.7</v>
+      </c>
+      <c r="W4" s="5">
+        <f>U4</f>
+        <v>0.7</v>
+      </c>
       <c r="X4" s="5">
         <f>U4</f>
         <v>0.7</v>
@@ -21008,6 +21104,10 @@
       <c r="V5">
         <v>0.1</v>
       </c>
+      <c r="W5" s="5">
+        <f>V5</f>
+        <v>0.1</v>
+      </c>
       <c r="X5" s="5">
         <f>V5</f>
         <v>0.1</v>
@@ -21212,6 +21312,10 @@
       <c r="V8">
         <v>0.5</v>
       </c>
+      <c r="W8" s="5">
+        <f>V8</f>
+        <v>0.5</v>
+      </c>
       <c r="X8" s="5">
         <f>V8</f>
         <v>0.5</v>
@@ -22002,6 +22106,14 @@
         <f>O20</f>
         <v>1.4</v>
       </c>
+      <c r="V20" s="5">
+        <f>O20</f>
+        <v>1.4</v>
+      </c>
+      <c r="W20" s="5">
+        <f>O20</f>
+        <v>1.4</v>
+      </c>
       <c r="X20" s="5">
         <f>O20</f>
         <v>1.4</v>
@@ -22314,6 +22426,10 @@
       <c r="V25">
         <v>30.3</v>
       </c>
+      <c r="W25" s="5">
+        <f>V25</f>
+        <v>30.3</v>
+      </c>
       <c r="X25">
         <v>21.8</v>
       </c>
@@ -22441,6 +22557,14 @@
         <v>0.5</v>
       </c>
       <c r="U27">
+        <v>0.5</v>
+      </c>
+      <c r="V27" s="5">
+        <f>U27</f>
+        <v>0.5</v>
+      </c>
+      <c r="W27" s="5">
+        <f>U27</f>
         <v>0.5</v>
       </c>
       <c r="X27" s="5">

</xml_diff>